<commit_message>
Eliminar archivo temporal de bloqueo de Excel
</commit_message>
<xml_diff>
--- a/01_datos/modificado/IE_SanLuis_v04.xlsx
+++ b/01_datos/modificado/IE_SanLuis_v04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\W11PRO\Downloads\IE-SanLuis-Portfolio\01_datos\modificado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F42F348-3926-453A-840F-9B91ECD45CEC}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C67D0F2-84DE-4C3E-B7DE-FA0F3E280D66}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -643,7 +643,310 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="32">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF5F5F5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -7026,8 +7329,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="2472334" y="9721786"/>
-              <a:ext cx="3743325" cy="3168000"/>
+              <a:off x="2469010" y="9876104"/>
+              <a:ext cx="3730410" cy="3214818"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7104,8 +7407,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6209338" y="9724667"/>
-              <a:ext cx="4559271" cy="702967"/>
+              <a:off x="6193099" y="9878985"/>
+              <a:ext cx="4539898" cy="715882"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7730,7 +8033,7 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C06B9CF3-B5DA-4E64-81A5-54220C2D645D}" name="TablaDinámica2" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A18:G30" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <location ref="A13:G25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -7891,16 +8194,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tbl_datos_base" displayName="tbl_datos_base" ref="A2:G12" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tbl_datos_base" displayName="tbl_datos_base" ref="A2:G12" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28">
   <autoFilter ref="A2:G12" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Código" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Departamento" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="1980" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="1991" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="2001" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="2010" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="2022" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Código" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Departamento" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="1980" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="1991" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="2001" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="2010" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="2022" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7913,47 +8216,47 @@
     <tableColumn id="1" xr3:uid="{779D6945-AD5E-45C6-9FED-6DF84B1D1D91}" name="Código"/>
     <tableColumn id="2" xr3:uid="{96B243D2-F081-43F7-B2AC-4670733E5D34}" name="Departamento"/>
     <tableColumn id="3" xr3:uid="{3286FD49-FC74-41CD-95B3-0BC34D94F4A5}" name="Año"/>
-    <tableColumn id="4" xr3:uid="{7C6DDE0F-DF73-43D8-886E-F795137ED3D9}" name="IE" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{7C6DDE0F-DF73-43D8-886E-F795137ED3D9}" name="IE" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B5DD205C-C525-48EA-9B11-D2B525172ED7}" name="Tabla3" displayName="Tabla3" ref="A3:J13" totalsRowShown="0" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B5DD205C-C525-48EA-9B11-D2B525172ED7}" name="Tabla3" displayName="Tabla3" ref="A3:J13" tableBorderDxfId="19">
   <autoFilter ref="A3:J13" xr:uid="{92801B63-9949-4FAD-A115-2BA00703E7C0}"/>
   <sortState ref="A4:I13">
     <sortCondition descending="1" ref="D4:D13"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{20DDF962-F49C-425A-ACBB-5D5495439CD6}" name="Código" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{20DDF962-F49C-425A-ACBB-5D5495439CD6}" name="Código" totalsRowLabel="Total" dataDxfId="16" totalsRowDxfId="0">
       <calculatedColumnFormula>'Datos base'!A4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{932355CE-4A7E-44CC-9979-D3C13AC77F08}" name="Departamento" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{932355CE-4A7E-44CC-9979-D3C13AC77F08}" name="Departamento" dataDxfId="15" totalsRowDxfId="1">
       <calculatedColumnFormula>'Datos base'!B4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F9C633E3-227E-41E1-9EFF-41246E37C3AC}" name="IE 2010" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{F9C633E3-227E-41E1-9EFF-41246E37C3AC}" name="IE 2010" dataDxfId="18" totalsRowDxfId="2">
       <calculatedColumnFormula>'Datos base'!F3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A469218B-F750-4ABF-9A56-4E7E021CA979}" name="IE 2022" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{A469218B-F750-4ABF-9A56-4E7E021CA979}" name="IE 2022" dataDxfId="17" totalsRowDxfId="3">
       <calculatedColumnFormula>'Datos base'!G3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{22AA691D-3291-4E94-99D0-ABF53B682F1C}" name="Var. absoluta_x000a_(2022−2010)" dataDxfId="5">
+    <tableColumn id="5" xr3:uid="{22AA691D-3291-4E94-99D0-ABF53B682F1C}" name="Var. absoluta_x000a_(2022−2010)" dataDxfId="14" totalsRowDxfId="4">
       <calculatedColumnFormula>D4-C4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E9249C1F-A735-4322-850B-BD7EAFB5ADC4}" name="Var. relativa_x000a_(%)" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{E9249C1F-A735-4322-850B-BD7EAFB5ADC4}" name="Var. relativa_x000a_(%)" dataDxfId="13" totalsRowDxfId="5">
       <calculatedColumnFormula>IFERROR((D4-C4)/C4*100,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{069C69A5-328B-4DE3-82FB-CEB3A0505D04}" name="Ranking IE_x000a_2022" dataDxfId="3">
+    <tableColumn id="7" xr3:uid="{069C69A5-328B-4DE3-82FB-CEB3A0505D04}" name="Ranking IE_x000a_2022" dataDxfId="12" totalsRowDxfId="6">
       <calculatedColumnFormula>RANK(D4,$D$4:$D$12,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A71D96E3-DFDA-4541-B5D5-C4E7F5E588E8}" name="Ranking Var._x000a_absoluta" dataDxfId="2">
+    <tableColumn id="8" xr3:uid="{A71D96E3-DFDA-4541-B5D5-C4E7F5E588E8}" name="Ranking Var._x000a_absoluta" dataDxfId="11" totalsRowDxfId="7">
       <calculatedColumnFormula>RANK(E4,$E$4:$E$12,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B21B4D9A-CBD5-44A2-BB6E-AA90D8B5E98C}" name="Referencia Provincial (IE = 47)" dataDxfId="1">
+    <tableColumn id="9" xr3:uid="{B21B4D9A-CBD5-44A2-BB6E-AA90D8B5E98C}" name="Referencia Provincial (IE = 47)" dataDxfId="10" totalsRowDxfId="8">
       <calculatedColumnFormula>47</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{480AE1C6-B89E-4484-AF9F-A34C4FFB092C}" name="Sobre IE Provincial (&gt; 47)" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{480AE1C6-B89E-4484-AF9F-A34C4FFB092C}" name="Sobre IE Provincial (&gt; 47)" totalsRowFunction="count" dataDxfId="9">
       <calculatedColumnFormula>IF(D4 &gt; 47, D4, NA())</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9326,7 +9629,7 @@
     <col min="5" max="6" width="14" style="10" customWidth="1"/>
     <col min="7" max="7" width="12" style="10" customWidth="1"/>
     <col min="8" max="8" width="15" style="10" customWidth="1"/>
-    <col min="9" max="9" width="30" style="26" customWidth="1"/>
+    <col min="9" max="9" width="33.28515625" style="26" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24" style="26" bestFit="1" customWidth="1"/>
   </cols>
@@ -9343,6 +9646,8 @@
       <c r="G1" s="38"/>
       <c r="H1" s="38"/>
       <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
     </row>
     <row r="2" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
@@ -9840,7 +10145,7 @@
   <mergeCells count="3">
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D12">
     <cfRule type="colorScale" priority="1">
@@ -9873,7 +10178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14D6844D-1525-4297-AA15-AD6A07CD63FF}">
-  <dimension ref="A3:L30"/>
+  <dimension ref="A3:L25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
@@ -10161,245 +10466,245 @@
         <v>36.04</v>
       </c>
     </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32">
+        <v>0</v>
+      </c>
+      <c r="D15" s="32">
+        <v>6</v>
+      </c>
+      <c r="E15" s="32">
+        <v>2</v>
+      </c>
+      <c r="F15" s="32">
+        <v>18</v>
+      </c>
+      <c r="G15" s="32"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32">
+        <v>11</v>
+      </c>
+      <c r="D16" s="32">
+        <v>12</v>
+      </c>
+      <c r="E16" s="32">
+        <v>6</v>
+      </c>
+      <c r="F16" s="32">
+        <v>11</v>
+      </c>
+      <c r="G16" s="32"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32">
+        <v>1</v>
+      </c>
+      <c r="D17" s="32">
+        <v>2</v>
+      </c>
+      <c r="E17" s="32">
+        <v>12</v>
+      </c>
+      <c r="F17" s="32">
+        <v>21</v>
+      </c>
+      <c r="G17" s="32"/>
+    </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="30" t="s">
-        <v>32</v>
-      </c>
+      <c r="A18" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="32"/>
+      <c r="C18" s="32">
+        <v>0</v>
+      </c>
+      <c r="D18" s="32">
+        <v>6</v>
+      </c>
+      <c r="E18" s="32">
+        <v>6</v>
+      </c>
+      <c r="F18" s="32">
+        <v>20</v>
+      </c>
+      <c r="G18" s="32"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="26" t="s">
+      <c r="A19" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="32"/>
+      <c r="C19" s="32">
+        <v>-3</v>
+      </c>
+      <c r="D19" s="32">
         <v>3</v>
       </c>
-      <c r="C19" s="26" t="s">
-        <v>4</v>
-      </c>
-      <c r="D19" s="26" t="s">
+      <c r="E19" s="32">
         <v>5</v>
       </c>
-      <c r="E19" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>31</v>
-      </c>
+      <c r="F19" s="32">
+        <v>13</v>
+      </c>
+      <c r="G19" s="32"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B20" s="32"/>
       <c r="C20" s="32">
+        <v>3</v>
+      </c>
+      <c r="D20" s="32">
         <v>0</v>
       </c>
-      <c r="D20" s="32">
+      <c r="E20" s="32">
         <v>6</v>
       </c>
-      <c r="E20" s="32">
-        <v>2</v>
-      </c>
       <c r="F20" s="32">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G20" s="32"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B21" s="32"/>
       <c r="C21" s="32">
-        <v>11</v>
+        <v>-7</v>
       </c>
       <c r="D21" s="32">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E21" s="32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F21" s="32">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G21" s="32"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B22" s="32"/>
       <c r="C22" s="32">
         <v>1</v>
       </c>
       <c r="D22" s="32">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E22" s="32">
         <v>12</v>
       </c>
       <c r="F22" s="32">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="G22" s="32"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B23" s="32"/>
       <c r="C23" s="32">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D23" s="32">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E23" s="32">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F23" s="32">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G23" s="32"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B24" s="32"/>
       <c r="C24" s="32">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="D24" s="32">
         <v>3</v>
       </c>
       <c r="E24" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" s="32">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G24" s="32"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="B25" s="32"/>
       <c r="C25" s="32">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D25" s="32">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="E25" s="32">
-        <v>6</v>
+        <v>73</v>
       </c>
       <c r="F25" s="32">
-        <v>10</v>
+        <v>166</v>
       </c>
       <c r="G25" s="32"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32">
-        <v>-7</v>
-      </c>
-      <c r="D26" s="32">
-        <v>2</v>
-      </c>
-      <c r="E26" s="32">
-        <v>7</v>
-      </c>
-      <c r="F26" s="32">
-        <v>17</v>
-      </c>
-      <c r="G26" s="32"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32">
-        <v>1</v>
-      </c>
-      <c r="D27" s="32">
-        <v>6</v>
-      </c>
-      <c r="E27" s="32">
-        <v>12</v>
-      </c>
-      <c r="F27" s="32">
-        <v>13</v>
-      </c>
-      <c r="G27" s="32"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32">
-        <v>12</v>
-      </c>
-      <c r="D28" s="32">
-        <v>3</v>
-      </c>
-      <c r="E28" s="32">
-        <v>11</v>
-      </c>
-      <c r="F28" s="32">
-        <v>27</v>
-      </c>
-      <c r="G28" s="32"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32">
-        <v>-4</v>
-      </c>
-      <c r="D29" s="32">
-        <v>3</v>
-      </c>
-      <c r="E29" s="32">
-        <v>6</v>
-      </c>
-      <c r="F29" s="32">
-        <v>16</v>
-      </c>
-      <c r="G29" s="32"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32">
-        <v>14</v>
-      </c>
-      <c r="D30" s="32">
-        <v>43</v>
-      </c>
-      <c r="E30" s="32">
-        <v>73</v>
-      </c>
-      <c r="F30" s="32">
-        <v>166</v>
-      </c>
-      <c r="G30" s="32"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>